<commit_message>
CI Reports [2026-07-02 20:36]: Login — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_02-Jul-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_02-Jul-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S39"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2727,9 +2727,70 @@
         <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
       </c>
     </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>02 Jul 2026</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Login</v>
+      </c>
+      <c r="C39" t="str">
+        <v>TC-LOGIN-017</v>
+      </c>
+      <c r="D39" t="str">
+        <v>SQL injection in username handled safely</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F39" t="str">
+        <v>API</v>
+      </c>
+      <c r="G39" t="str">
+        <v>High</v>
+      </c>
+      <c r="H39" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I39" t="str">
+        <v>BUG-LOGIN-038</v>
+      </c>
+      <c r="J39" t="str">
+        <v>SQL injection in username handled safely</v>
+      </c>
+      <c r="K39" t="str">
+        <v>High</v>
+      </c>
+      <c r="L39" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M39" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P39" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter ' OR 1=1 -- as username
+2. Click Sign In (JS click — allow 4–6 s)
+3. Check URL, page title, and any error messages for SQL bypass or 500</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>SQL injection rejected; stays on /Account/Login; no SQL error exposed; authentication not bypassed</v>
+      </c>
+      <c r="R39" t="str">
+        <v>Error: expect(page).toHaveURL(expected) failed Expected pattern: /Login/ Received string: "" Timeout: 5000ms Call log: - Expect "toHaveURL" with timeout 5000ms - waiting for" http://customerportal.dev-ts.online/Account/Login" navigation to finish...</v>
+      </c>
+      <c r="S39" t="str">
+        <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>